<commit_message>
Update TEAM_1_Project Status Report.xlsx
</commit_message>
<xml_diff>
--- a/Docs/report/TEAM_1_Project Status Report.xlsx
+++ b/Docs/report/TEAM_1_Project Status Report.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QA-Project\QA-project-tool\Docs\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A5EDD5-D2BB-4690-94FF-73CBD7E6F336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3539A87F-D063-47CA-9A59-8F5C9C2FFA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Release#1" sheetId="1" r:id="rId1"/>
     <sheet name="Release#2" sheetId="2" r:id="rId2"/>
     <sheet name="Release#3" sheetId="4" r:id="rId3"/>
     <sheet name="Release#4" sheetId="3" r:id="rId4"/>
+    <sheet name="Release#5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
-    <pivotCache cacheId="1" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,14 +35,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="3Ua4wsPVU2+OjJeWbmtYzx5bg+lUiDntYAmcCMaFM74="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="3Ua4wsPVU2+OjJeWbmtYzx5bg+lUiDntYAmcCMaFM74="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="128">
   <si>
     <t>Day</t>
   </si>
@@ -425,6 +426,18 @@
   </si>
   <si>
     <t>lack of team members due to illnes</t>
+  </si>
+  <si>
+    <t>backend development1</t>
+  </si>
+  <si>
+    <t>backend development2</t>
+  </si>
+  <si>
+    <t>continue front development 1</t>
+  </si>
+  <si>
+    <t>continue front development 2</t>
   </si>
 </sst>
 </file>
@@ -868,7 +881,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1088,25 +1101,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1120,12 +1131,26 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3166,6 +3191,734 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-6FE9-479D-AF38-9962CB2B10FC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="2028298865"/>
+        <c:axId val="517339348"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="2028298865"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="900" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="517339348"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="517339348"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="900" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2028298865"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr sz="900" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Planned</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="4285F4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Release#5'!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Release#5'!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A9FB-4840-8A6B-081AD16780F7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Consumed</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="EA4335"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Release#5'!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Release#5'!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A9FB-4840-8A6B-081AD16780F7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="759985173"/>
+        <c:axId val="398362538"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="759985173"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="398362538"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="398362538"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="759985173"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[TEAM_1_Project Status Report.xlsx]Release#5!Release#3</c:name>
+    <c:fmtId val="2"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.4701895161049923E-2"/>
+          <c:y val="5.8479532163742687E-2"/>
+          <c:w val="0.74860068676487246"/>
+          <c:h val="0.79150097465886937"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Release#5'!$Q$4:$Q$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Hours</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Release#5'!$P$6:$P$11</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>abdalrahman</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>alaaa</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>alhussin</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>nabil</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>zahraan</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Release#5'!$Q$6:$Q$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-27E8-4D4C-BC0C-4E8D0968ACC2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Release#5'!$R$4:$R$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Done</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Release#5'!$P$6:$P$11</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>abdalrahman</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>alaaa</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>alhussin</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>nabil</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>zahraan</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Release#5'!$R$6:$R$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-27E8-4D4C-BC0C-4E8D0968ACC2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3530,6 +4283,77 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B4FB73D-306B-4107-B738-2493F758EDC5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1251857</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>217714</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7549243" cy="2677886"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33F76CC8-30FA-4124-99D7-59CAFB430D91}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>4118</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>98338</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6709720" cy="3257550"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{775B1C2F-8CB5-4C3E-9C61-C9C624F147F4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4116,6 +4940,110 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C4D24A4A-83E6-4F38-BF99-7949CBE850DD}" name="Release#3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="7" compact="0" compactData="0" chartFormat="3">
+  <location ref="P4:R11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="5">
+    <pivotField name="Deliverable" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="% Completed" compact="0" numFmtId="9" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="Comments" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="6">
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField name="Done" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Hours" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Done" fld="4" baseField="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="1" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="1" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -4498,15 +5426,15 @@
       <c r="I11" s="10"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="89" t="s">
+      <c r="A12" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="90"/>
-      <c r="C12" s="90"/>
-      <c r="D12" s="90"/>
-      <c r="E12" s="90"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="91"/>
+      <c r="B12" s="94"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="94"/>
+      <c r="E12" s="94"/>
+      <c r="F12" s="94"/>
+      <c r="G12" s="95"/>
       <c r="I12" s="10"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4756,15 +5684,15 @@
       <c r="I26" s="10"/>
     </row>
     <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="89" t="s">
+      <c r="A27" s="93" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="90"/>
-      <c r="C27" s="90"/>
-      <c r="D27" s="90"/>
-      <c r="E27" s="90"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="91"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="94"/>
+      <c r="F27" s="94"/>
+      <c r="G27" s="95"/>
       <c r="I27" s="10"/>
     </row>
     <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7242,15 +8170,15 @@
       <c r="I12" s="10"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="89" t="s">
+      <c r="A13" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="91"/>
+      <c r="B13" s="94"/>
+      <c r="C13" s="94"/>
+      <c r="D13" s="94"/>
+      <c r="E13" s="94"/>
+      <c r="F13" s="94"/>
+      <c r="G13" s="95"/>
       <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7332,15 +8260,15 @@
       <c r="I20" s="10"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="89" t="s">
+      <c r="A21" s="93" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="90"/>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="91"/>
+      <c r="B21" s="94"/>
+      <c r="C21" s="94"/>
+      <c r="D21" s="94"/>
+      <c r="E21" s="94"/>
+      <c r="F21" s="94"/>
+      <c r="G21" s="95"/>
       <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9998,15 +10926,15 @@
       </c>
     </row>
     <row r="12" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="98" t="s">
+      <c r="A12" s="96" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="99"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="99"/>
-      <c r="F12" s="99"/>
-      <c r="G12" s="99"/>
+      <c r="B12" s="97"/>
+      <c r="C12" s="97"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="97"/>
+      <c r="F12" s="97"/>
+      <c r="G12" s="97"/>
       <c r="I12" s="35" t="s">
         <v>82</v>
       </c>
@@ -10401,15 +11329,15 @@
       </c>
     </row>
     <row r="28" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="98" t="s">
+      <c r="A28" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="99"/>
-      <c r="C28" s="99"/>
-      <c r="D28" s="99"/>
-      <c r="E28" s="99"/>
-      <c r="F28" s="99"/>
-      <c r="G28" s="99"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
       <c r="I28" s="35" t="s">
         <v>66</v>
       </c>
@@ -10665,7 +11593,7 @@
       <c r="B43" s="21"/>
       <c r="C43" s="21"/>
       <c r="D43" s="21"/>
-      <c r="N43" s="100">
+      <c r="N43" s="98">
         <v>1</v>
       </c>
       <c r="O43" s="25">
@@ -10679,7 +11607,7 @@
         <f>VLOOKUP(P43,$I$2:$L$36,3,FALSE)</f>
         <v>nabil</v>
       </c>
-      <c r="R43" s="95">
+      <c r="R43" s="101">
         <f>SUM(O43:O50)</f>
         <v>24</v>
       </c>
@@ -10689,7 +11617,7 @@
       <c r="B44" s="21"/>
       <c r="C44" s="21"/>
       <c r="D44" s="21"/>
-      <c r="N44" s="101"/>
+      <c r="N44" s="99"/>
       <c r="O44" s="25">
         <f t="shared" ref="O44:O71" si="0">VLOOKUP(P44,$I$3:$L$36,4,FALSE)</f>
         <v>3</v>
@@ -10701,14 +11629,14 @@
         <f t="shared" ref="Q44:Q71" si="1">VLOOKUP(P44,$I$3:$L$36,3,FALSE)</f>
         <v>alaaa</v>
       </c>
-      <c r="R44" s="95"/>
+      <c r="R44" s="101"/>
     </row>
     <row r="45" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21"/>
       <c r="B45" s="21"/>
       <c r="C45" s="21"/>
       <c r="D45" s="21"/>
-      <c r="N45" s="101"/>
+      <c r="N45" s="99"/>
       <c r="O45" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10720,14 +11648,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R45" s="95"/>
+      <c r="R45" s="101"/>
     </row>
     <row r="46" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="21"/>
       <c r="B46" s="21"/>
       <c r="C46" s="21"/>
       <c r="D46" s="21"/>
-      <c r="N46" s="101"/>
+      <c r="N46" s="99"/>
       <c r="O46" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10739,14 +11667,14 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R46" s="95"/>
+      <c r="R46" s="101"/>
     </row>
     <row r="47" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="21"/>
       <c r="B47" s="21"/>
       <c r="C47" s="21"/>
       <c r="D47" s="21"/>
-      <c r="N47" s="101"/>
+      <c r="N47" s="99"/>
       <c r="O47" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10758,14 +11686,14 @@
         <f t="shared" si="1"/>
         <v>nabil</v>
       </c>
-      <c r="R47" s="95"/>
+      <c r="R47" s="101"/>
     </row>
     <row r="48" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="21"/>
       <c r="B48" s="21"/>
       <c r="C48" s="21"/>
       <c r="D48" s="21"/>
-      <c r="N48" s="101"/>
+      <c r="N48" s="99"/>
       <c r="O48" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10777,14 +11705,14 @@
         <f t="shared" si="1"/>
         <v>nabil</v>
       </c>
-      <c r="R48" s="95"/>
+      <c r="R48" s="101"/>
     </row>
     <row r="49" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="21"/>
       <c r="B49" s="21"/>
       <c r="C49" s="21"/>
       <c r="D49" s="21"/>
-      <c r="N49" s="101"/>
+      <c r="N49" s="99"/>
       <c r="O49" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10796,14 +11724,14 @@
         <f t="shared" si="1"/>
         <v>Boda</v>
       </c>
-      <c r="R49" s="95"/>
+      <c r="R49" s="101"/>
     </row>
     <row r="50" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="21"/>
       <c r="B50" s="21"/>
       <c r="C50" s="21"/>
       <c r="D50" s="21"/>
-      <c r="N50" s="102"/>
+      <c r="N50" s="100"/>
       <c r="O50" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -10815,14 +11743,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R50" s="103"/>
+      <c r="R50" s="102"/>
     </row>
     <row r="51" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="21"/>
       <c r="B51" s="21"/>
       <c r="C51" s="21"/>
       <c r="D51" s="21"/>
-      <c r="N51" s="100">
+      <c r="N51" s="98">
         <v>2</v>
       </c>
       <c r="O51" s="25">
@@ -10836,7 +11764,7 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R51" s="104">
+      <c r="R51" s="103">
         <f>SUM(O51:O52)</f>
         <v>4</v>
       </c>
@@ -10846,7 +11774,7 @@
       <c r="B52" s="21"/>
       <c r="C52" s="21"/>
       <c r="D52" s="21"/>
-      <c r="N52" s="101"/>
+      <c r="N52" s="99"/>
       <c r="O52" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -10858,7 +11786,7 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R52" s="104"/>
+      <c r="R52" s="103"/>
     </row>
     <row r="53" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="21"/>
@@ -10889,7 +11817,7 @@
       <c r="B54" s="21"/>
       <c r="C54" s="21"/>
       <c r="D54" s="21"/>
-      <c r="N54" s="92">
+      <c r="N54" s="104">
         <v>4</v>
       </c>
       <c r="O54" s="25">
@@ -10903,7 +11831,7 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R54" s="94">
+      <c r="R54" s="106">
         <f>SUM(O54:O61)</f>
         <v>8</v>
       </c>
@@ -10913,7 +11841,7 @@
       <c r="B55" s="21"/>
       <c r="C55" s="21"/>
       <c r="D55" s="21"/>
-      <c r="N55" s="93"/>
+      <c r="N55" s="105"/>
       <c r="O55" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -10925,14 +11853,14 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R55" s="95"/>
+      <c r="R55" s="101"/>
     </row>
     <row r="56" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="21"/>
       <c r="B56" s="21"/>
       <c r="C56" s="21"/>
       <c r="D56" s="21"/>
-      <c r="N56" s="93"/>
+      <c r="N56" s="105"/>
       <c r="O56" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -10944,14 +11872,14 @@
         <f t="shared" si="1"/>
         <v>alaaa</v>
       </c>
-      <c r="R56" s="95"/>
+      <c r="R56" s="101"/>
     </row>
     <row r="57" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="21"/>
       <c r="B57" s="21"/>
       <c r="C57" s="21"/>
       <c r="D57" s="21"/>
-      <c r="N57" s="93"/>
+      <c r="N57" s="105"/>
       <c r="O57" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -10963,14 +11891,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R57" s="95"/>
+      <c r="R57" s="101"/>
     </row>
     <row r="58" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21"/>
       <c r="B58" s="21"/>
       <c r="C58" s="21"/>
       <c r="D58" s="21"/>
-      <c r="N58" s="93"/>
+      <c r="N58" s="105"/>
       <c r="O58" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -10982,14 +11910,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R58" s="95"/>
+      <c r="R58" s="101"/>
     </row>
     <row r="59" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="21"/>
       <c r="B59" s="21"/>
       <c r="C59" s="21"/>
       <c r="D59" s="21"/>
-      <c r="N59" s="93"/>
+      <c r="N59" s="105"/>
       <c r="O59" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -11001,14 +11929,14 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R59" s="95"/>
+      <c r="R59" s="101"/>
     </row>
     <row r="60" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="21"/>
       <c r="B60" s="21"/>
       <c r="C60" s="21"/>
       <c r="D60" s="21"/>
-      <c r="N60" s="93"/>
+      <c r="N60" s="105"/>
       <c r="O60" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -11020,14 +11948,14 @@
         <f t="shared" si="1"/>
         <v>alaaa</v>
       </c>
-      <c r="R60" s="95"/>
+      <c r="R60" s="101"/>
     </row>
     <row r="61" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="21"/>
       <c r="B61" s="21"/>
       <c r="C61" s="21"/>
       <c r="D61" s="21"/>
-      <c r="N61" s="93"/>
+      <c r="N61" s="105"/>
       <c r="O61" s="25">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -11039,14 +11967,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R61" s="96"/>
+      <c r="R61" s="107"/>
     </row>
     <row r="62" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="21"/>
       <c r="B62" s="21"/>
       <c r="C62" s="21"/>
       <c r="D62" s="21"/>
-      <c r="N62" s="92">
+      <c r="N62" s="104">
         <v>5</v>
       </c>
       <c r="O62" s="25">
@@ -11060,7 +11988,7 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R62" s="94">
+      <c r="R62" s="106">
         <f>SUM(O62:O66)</f>
         <v>12</v>
       </c>
@@ -11070,7 +11998,7 @@
       <c r="B63" s="21"/>
       <c r="C63" s="21"/>
       <c r="D63" s="21"/>
-      <c r="N63" s="93"/>
+      <c r="N63" s="105"/>
       <c r="O63" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11082,14 +12010,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R63" s="93"/>
+      <c r="R63" s="105"/>
     </row>
     <row r="64" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="21"/>
       <c r="B64" s="21"/>
       <c r="C64" s="21"/>
       <c r="D64" s="21"/>
-      <c r="N64" s="93"/>
+      <c r="N64" s="105"/>
       <c r="O64" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11101,14 +12029,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R64" s="93"/>
+      <c r="R64" s="105"/>
     </row>
     <row r="65" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="21"/>
       <c r="B65" s="21"/>
       <c r="C65" s="21"/>
       <c r="D65" s="21"/>
-      <c r="N65" s="93"/>
+      <c r="N65" s="105"/>
       <c r="O65" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11120,14 +12048,14 @@
         <f t="shared" si="1"/>
         <v>alaaa</v>
       </c>
-      <c r="R65" s="93"/>
+      <c r="R65" s="105"/>
     </row>
     <row r="66" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="21"/>
       <c r="B66" s="21"/>
       <c r="C66" s="21"/>
       <c r="D66" s="21"/>
-      <c r="N66" s="97"/>
+      <c r="N66" s="108"/>
       <c r="O66" s="25">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -11139,14 +12067,14 @@
         <f t="shared" si="1"/>
         <v>nabil</v>
       </c>
-      <c r="R66" s="97"/>
+      <c r="R66" s="108"/>
     </row>
     <row r="67" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="21"/>
       <c r="B67" s="21"/>
       <c r="C67" s="21"/>
       <c r="D67" s="21"/>
-      <c r="N67" s="92">
+      <c r="N67" s="104">
         <v>6</v>
       </c>
       <c r="O67" s="25">
@@ -11160,7 +12088,7 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R67" s="94">
+      <c r="R67" s="106">
         <f>SUM(O67:O71)</f>
         <v>12</v>
       </c>
@@ -11170,7 +12098,7 @@
       <c r="B68" s="21"/>
       <c r="C68" s="21"/>
       <c r="D68" s="21"/>
-      <c r="N68" s="93"/>
+      <c r="N68" s="105"/>
       <c r="O68" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11182,14 +12110,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R68" s="93"/>
+      <c r="R68" s="105"/>
     </row>
     <row r="69" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="21"/>
       <c r="B69" s="21"/>
       <c r="C69" s="21"/>
       <c r="D69" s="21"/>
-      <c r="N69" s="93"/>
+      <c r="N69" s="105"/>
       <c r="O69" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11201,14 +12129,14 @@
         <f t="shared" si="1"/>
         <v>alaaa</v>
       </c>
-      <c r="R69" s="93"/>
+      <c r="R69" s="105"/>
     </row>
     <row r="70" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="21"/>
       <c r="B70" s="21"/>
       <c r="C70" s="21"/>
       <c r="D70" s="21"/>
-      <c r="N70" s="93"/>
+      <c r="N70" s="105"/>
       <c r="O70" s="25">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -11220,14 +12148,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R70" s="93"/>
+      <c r="R70" s="105"/>
     </row>
     <row r="71" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="21"/>
       <c r="B71" s="21"/>
       <c r="C71" s="21"/>
       <c r="D71" s="21"/>
-      <c r="N71" s="97"/>
+      <c r="N71" s="108"/>
       <c r="O71" s="25">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -11239,7 +12167,7 @@
         <f t="shared" si="1"/>
         <v>nabil</v>
       </c>
-      <c r="R71" s="97"/>
+      <c r="R71" s="108"/>
     </row>
     <row r="72" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="21"/>
@@ -12211,18 +13139,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="N54:N61"/>
+    <mergeCell ref="R54:R61"/>
+    <mergeCell ref="N62:N66"/>
+    <mergeCell ref="R62:R66"/>
+    <mergeCell ref="N67:N71"/>
+    <mergeCell ref="R67:R71"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="N43:N50"/>
     <mergeCell ref="R43:R50"/>
     <mergeCell ref="N51:N52"/>
     <mergeCell ref="R51:R52"/>
-    <mergeCell ref="N54:N61"/>
-    <mergeCell ref="R54:R61"/>
-    <mergeCell ref="N62:N66"/>
-    <mergeCell ref="R62:R66"/>
-    <mergeCell ref="N67:N71"/>
-    <mergeCell ref="R67:R71"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F14:F25 F30:F40" xr:uid="{AFC4AC33-7B9C-40BD-80E0-C1F9CEEBC5BF}">
@@ -12616,15 +13544,15 @@
       </c>
     </row>
     <row r="12" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="98" t="s">
+      <c r="A12" s="96" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="99"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="99"/>
-      <c r="F12" s="99"/>
-      <c r="G12" s="99"/>
+      <c r="B12" s="97"/>
+      <c r="C12" s="97"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="97"/>
+      <c r="F12" s="97"/>
+      <c r="G12" s="97"/>
       <c r="I12" s="35" t="s">
         <v>121</v>
       </c>
@@ -12873,15 +13801,15 @@
       <c r="M27" s="22"/>
     </row>
     <row r="28" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="98" t="s">
+      <c r="A28" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="99"/>
-      <c r="C28" s="99"/>
-      <c r="D28" s="99"/>
-      <c r="E28" s="99"/>
-      <c r="F28" s="99"/>
-      <c r="G28" s="99"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
       <c r="I28" s="35"/>
       <c r="J28" s="43"/>
       <c r="K28" s="43"/>
@@ -13105,7 +14033,7 @@
       <c r="B43" s="21"/>
       <c r="C43" s="21"/>
       <c r="D43" s="21"/>
-      <c r="N43" s="100">
+      <c r="N43" s="98">
         <v>1</v>
       </c>
       <c r="O43" s="25">
@@ -13119,7 +14047,7 @@
         <f>VLOOKUP(P43,$I$2:$L$36,3,FALSE)</f>
         <v>nabil</v>
       </c>
-      <c r="R43" s="95">
+      <c r="R43" s="101">
         <f>SUM(O43:O47)</f>
         <v>15</v>
       </c>
@@ -13129,7 +14057,7 @@
       <c r="B44" s="21"/>
       <c r="C44" s="21"/>
       <c r="D44" s="21"/>
-      <c r="N44" s="101"/>
+      <c r="N44" s="99"/>
       <c r="O44" s="25">
         <f t="shared" ref="O44:O68" si="0">VLOOKUP(P44,$I$3:$L$36,4,FALSE)</f>
         <v>3</v>
@@ -13141,14 +14069,14 @@
         <f t="shared" ref="Q44:Q68" si="1">VLOOKUP(P44,$I$3:$L$36,3,FALSE)</f>
         <v>alaaa</v>
       </c>
-      <c r="R44" s="95"/>
+      <c r="R44" s="101"/>
     </row>
     <row r="45" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21"/>
       <c r="B45" s="21"/>
       <c r="C45" s="21"/>
       <c r="D45" s="21"/>
-      <c r="N45" s="101"/>
+      <c r="N45" s="99"/>
       <c r="O45" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -13160,14 +14088,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R45" s="95"/>
+      <c r="R45" s="101"/>
     </row>
     <row r="46" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="21"/>
       <c r="B46" s="21"/>
       <c r="C46" s="21"/>
       <c r="D46" s="21"/>
-      <c r="N46" s="101"/>
+      <c r="N46" s="99"/>
       <c r="O46" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -13179,14 +14107,14 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R46" s="95"/>
+      <c r="R46" s="101"/>
     </row>
     <row r="47" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="21"/>
       <c r="B47" s="21"/>
       <c r="C47" s="21"/>
       <c r="D47" s="21"/>
-      <c r="N47" s="101"/>
+      <c r="N47" s="99"/>
       <c r="O47" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -13198,14 +14126,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R47" s="95"/>
+      <c r="R47" s="101"/>
     </row>
     <row r="48" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="21"/>
       <c r="B48" s="21"/>
       <c r="C48" s="21"/>
       <c r="D48" s="21"/>
-      <c r="N48" s="100">
+      <c r="N48" s="98">
         <v>2</v>
       </c>
       <c r="O48" s="25">
@@ -13219,7 +14147,7 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R48" s="104">
+      <c r="R48" s="103">
         <f>SUM(O48:O49)</f>
         <v>6</v>
       </c>
@@ -13229,7 +14157,7 @@
       <c r="B49" s="21"/>
       <c r="C49" s="21"/>
       <c r="D49" s="21"/>
-      <c r="N49" s="101"/>
+      <c r="N49" s="99"/>
       <c r="O49" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -13241,7 +14169,7 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R49" s="104"/>
+      <c r="R49" s="103"/>
     </row>
     <row r="50" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="21"/>
@@ -13269,7 +14197,7 @@
       <c r="B51" s="21"/>
       <c r="C51" s="21"/>
       <c r="D51" s="21"/>
-      <c r="N51" s="92">
+      <c r="N51" s="104">
         <v>4</v>
       </c>
       <c r="O51" s="25" t="e">
@@ -13281,7 +14209,7 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R51" s="94">
+      <c r="R51" s="106">
         <v>0</v>
       </c>
     </row>
@@ -13290,7 +14218,7 @@
       <c r="B52" s="21"/>
       <c r="C52" s="21"/>
       <c r="D52" s="21"/>
-      <c r="N52" s="93"/>
+      <c r="N52" s="105"/>
       <c r="O52" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13300,14 +14228,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R52" s="95"/>
+      <c r="R52" s="101"/>
     </row>
     <row r="53" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="21"/>
       <c r="B53" s="21"/>
       <c r="C53" s="21"/>
       <c r="D53" s="21"/>
-      <c r="N53" s="93"/>
+      <c r="N53" s="105"/>
       <c r="O53" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13317,14 +14245,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R53" s="95"/>
+      <c r="R53" s="101"/>
     </row>
     <row r="54" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="21"/>
       <c r="B54" s="21"/>
       <c r="C54" s="21"/>
       <c r="D54" s="21"/>
-      <c r="N54" s="93"/>
+      <c r="N54" s="105"/>
       <c r="O54" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13334,14 +14262,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R54" s="95"/>
+      <c r="R54" s="101"/>
     </row>
     <row r="55" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="21"/>
       <c r="B55" s="21"/>
       <c r="C55" s="21"/>
       <c r="D55" s="21"/>
-      <c r="N55" s="93"/>
+      <c r="N55" s="105"/>
       <c r="O55" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13351,14 +14279,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R55" s="95"/>
+      <c r="R55" s="101"/>
     </row>
     <row r="56" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="21"/>
       <c r="B56" s="21"/>
       <c r="C56" s="21"/>
       <c r="D56" s="21"/>
-      <c r="N56" s="93"/>
+      <c r="N56" s="105"/>
       <c r="O56" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13368,14 +14296,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R56" s="95"/>
+      <c r="R56" s="101"/>
     </row>
     <row r="57" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="21"/>
       <c r="B57" s="21"/>
       <c r="C57" s="21"/>
       <c r="D57" s="21"/>
-      <c r="N57" s="93"/>
+      <c r="N57" s="105"/>
       <c r="O57" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13385,14 +14313,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R57" s="95"/>
+      <c r="R57" s="101"/>
     </row>
     <row r="58" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21"/>
       <c r="B58" s="21"/>
       <c r="C58" s="21"/>
       <c r="D58" s="21"/>
-      <c r="N58" s="93"/>
+      <c r="N58" s="105"/>
       <c r="O58" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13402,14 +14330,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R58" s="96"/>
+      <c r="R58" s="107"/>
     </row>
     <row r="59" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="21"/>
       <c r="B59" s="21"/>
       <c r="C59" s="21"/>
       <c r="D59" s="21"/>
-      <c r="N59" s="92">
+      <c r="N59" s="104">
         <v>5</v>
       </c>
       <c r="O59" s="25" t="e">
@@ -13421,7 +14349,7 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R59" s="94">
+      <c r="R59" s="106">
         <v>0</v>
       </c>
     </row>
@@ -13430,7 +14358,7 @@
       <c r="B60" s="21"/>
       <c r="C60" s="21"/>
       <c r="D60" s="21"/>
-      <c r="N60" s="93"/>
+      <c r="N60" s="105"/>
       <c r="O60" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13440,14 +14368,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R60" s="93"/>
+      <c r="R60" s="105"/>
     </row>
     <row r="61" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="21"/>
       <c r="B61" s="21"/>
       <c r="C61" s="21"/>
       <c r="D61" s="21"/>
-      <c r="N61" s="93"/>
+      <c r="N61" s="105"/>
       <c r="O61" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13457,14 +14385,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R61" s="93"/>
+      <c r="R61" s="105"/>
     </row>
     <row r="62" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="21"/>
       <c r="B62" s="21"/>
       <c r="C62" s="21"/>
       <c r="D62" s="21"/>
-      <c r="N62" s="93"/>
+      <c r="N62" s="105"/>
       <c r="O62" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13474,14 +14402,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R62" s="93"/>
+      <c r="R62" s="105"/>
     </row>
     <row r="63" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="21"/>
       <c r="B63" s="21"/>
       <c r="C63" s="21"/>
       <c r="D63" s="21"/>
-      <c r="N63" s="97"/>
+      <c r="N63" s="108"/>
       <c r="O63" s="25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
@@ -13491,14 +14419,14 @@
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R63" s="97"/>
+      <c r="R63" s="108"/>
     </row>
     <row r="64" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="21"/>
       <c r="B64" s="21"/>
       <c r="C64" s="21"/>
       <c r="D64" s="21"/>
-      <c r="N64" s="92">
+      <c r="N64" s="104">
         <v>6</v>
       </c>
       <c r="O64" s="25">
@@ -13512,7 +14440,7 @@
         <f t="shared" si="1"/>
         <v>alaaa</v>
       </c>
-      <c r="R64" s="94">
+      <c r="R64" s="106">
         <f>SUM(O64:O68)</f>
         <v>29</v>
       </c>
@@ -13522,7 +14450,7 @@
       <c r="B65" s="21"/>
       <c r="C65" s="21"/>
       <c r="D65" s="21"/>
-      <c r="N65" s="93"/>
+      <c r="N65" s="105"/>
       <c r="O65" s="25">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -13534,14 +14462,14 @@
         <f t="shared" si="1"/>
         <v>abdalrahman</v>
       </c>
-      <c r="R65" s="93"/>
+      <c r="R65" s="105"/>
     </row>
     <row r="66" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="21"/>
       <c r="B66" s="21"/>
       <c r="C66" s="21"/>
       <c r="D66" s="21"/>
-      <c r="N66" s="93"/>
+      <c r="N66" s="105"/>
       <c r="O66" s="25">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -13553,14 +14481,14 @@
         <f t="shared" si="1"/>
         <v>alhussin</v>
       </c>
-      <c r="R66" s="93"/>
+      <c r="R66" s="105"/>
     </row>
     <row r="67" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="21"/>
       <c r="B67" s="21"/>
       <c r="C67" s="21"/>
       <c r="D67" s="21"/>
-      <c r="N67" s="93"/>
+      <c r="N67" s="105"/>
       <c r="O67" s="25">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -13572,14 +14500,14 @@
         <f t="shared" si="1"/>
         <v>zahraan</v>
       </c>
-      <c r="R67" s="93"/>
+      <c r="R67" s="105"/>
     </row>
     <row r="68" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="21"/>
       <c r="B68" s="21"/>
       <c r="C68" s="21"/>
       <c r="D68" s="21"/>
-      <c r="N68" s="97"/>
+      <c r="N68" s="108"/>
       <c r="O68" s="25">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -13591,7 +14519,7 @@
         <f t="shared" si="1"/>
         <v>nabil</v>
       </c>
-      <c r="R68" s="97"/>
+      <c r="R68" s="108"/>
     </row>
     <row r="69" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="21"/>
@@ -14563,6 +15491,9 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="R51:R58"/>
+    <mergeCell ref="R59:R63"/>
     <mergeCell ref="R64:R68"/>
     <mergeCell ref="N51:N58"/>
     <mergeCell ref="N59:N63"/>
@@ -14572,9 +15503,6 @@
     <mergeCell ref="R48:R49"/>
     <mergeCell ref="R43:R47"/>
     <mergeCell ref="N43:N47"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="R51:R58"/>
-    <mergeCell ref="R59:R63"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <dataValidations count="1">
@@ -14586,4 +15514,2281 @@
   <pageSetup orientation="portrait"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FB87AA-73A7-447D-A9F5-CCC196DD52C8}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:AB228"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="25.8" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.77734375" style="20" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="20" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" style="20" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="73.44140625" style="20" customWidth="1"/>
+    <col min="6" max="6" width="10" style="20" customWidth="1"/>
+    <col min="7" max="7" width="60.77734375" style="20" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="20"/>
+    <col min="9" max="9" width="59.44140625" style="20" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="20" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" style="20" customWidth="1"/>
+    <col min="12" max="13" width="12.6640625" style="20"/>
+    <col min="14" max="14" width="16.109375" style="20" customWidth="1"/>
+    <col min="15" max="15" width="8.33203125" style="20" customWidth="1"/>
+    <col min="16" max="16" width="47.109375" style="20" customWidth="1"/>
+    <col min="17" max="17" width="27" style="20" customWidth="1"/>
+    <col min="18" max="18" width="23.5546875" style="20" customWidth="1"/>
+    <col min="19" max="19" width="12.6640625" style="20"/>
+    <col min="20" max="20" width="8.88671875" style="20" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" style="20"/>
+    <col min="22" max="22" width="64.44140625" style="20" customWidth="1"/>
+    <col min="23" max="24" width="12.6640625" style="20"/>
+    <col min="25" max="25" width="75" style="20" customWidth="1"/>
+    <col min="26" max="16384" width="12.6640625" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="91" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="91" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="76" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="91" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="91" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" s="91" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="66">
+        <v>1</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="73">
+        <v>50</v>
+      </c>
+      <c r="I2" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" s="43">
+        <v>1</v>
+      </c>
+      <c r="K2" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="L2" s="72">
+        <v>3</v>
+      </c>
+      <c r="M2" s="71"/>
+    </row>
+    <row r="3" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="66">
+        <v>2</v>
+      </c>
+      <c r="B3" s="74"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="21"/>
+      <c r="I3" s="35" t="s">
+        <v>124</v>
+      </c>
+      <c r="J3" s="43">
+        <v>0</v>
+      </c>
+      <c r="K3" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="22">
+        <v>8</v>
+      </c>
+      <c r="M3" s="22"/>
+    </row>
+    <row r="4" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="66">
+        <v>3</v>
+      </c>
+      <c r="B4" s="74"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="21"/>
+      <c r="I4" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="J4" s="43">
+        <v>0</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="L4" s="22">
+        <v>8</v>
+      </c>
+      <c r="M4" s="22"/>
+      <c r="P4" s="77"/>
+      <c r="Q4" s="77" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4" s="79"/>
+    </row>
+    <row r="5" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="66">
+        <v>4</v>
+      </c>
+      <c r="B5" s="74"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="21"/>
+      <c r="I5" s="35" t="s">
+        <v>126</v>
+      </c>
+      <c r="J5" s="43">
+        <v>1</v>
+      </c>
+      <c r="K5" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="L5" s="22">
+        <v>2</v>
+      </c>
+      <c r="M5" s="22"/>
+      <c r="P5" s="77" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q5" s="77" t="s">
+        <v>108</v>
+      </c>
+      <c r="R5" s="80" t="s">
+        <v>107</v>
+      </c>
+      <c r="AB5" s="69"/>
+    </row>
+    <row r="6" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="66">
+        <v>5</v>
+      </c>
+      <c r="B6" s="74"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="21"/>
+      <c r="I6" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="J6" s="43">
+        <v>1</v>
+      </c>
+      <c r="K6" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="L6" s="22">
+        <v>2</v>
+      </c>
+      <c r="M6" s="22"/>
+      <c r="P6" s="77" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q6" s="81">
+        <v>11</v>
+      </c>
+      <c r="R6" s="82">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="66">
+        <v>6</v>
+      </c>
+      <c r="B7" s="65"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="21"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="43">
+        <v>1</v>
+      </c>
+      <c r="K7" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="P7" s="83" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q7" s="84">
+        <v>11</v>
+      </c>
+      <c r="R7" s="85">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="43">
+        <v>1</v>
+      </c>
+      <c r="K8" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="P8" s="83" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q8" s="84">
+        <v>11</v>
+      </c>
+      <c r="R8" s="85">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="43">
+        <v>1</v>
+      </c>
+      <c r="K9" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="P9" s="83" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q9" s="84">
+        <v>6</v>
+      </c>
+      <c r="R9" s="85">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="43">
+        <v>1</v>
+      </c>
+      <c r="K10" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="P10" s="83" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q10" s="84">
+        <v>11</v>
+      </c>
+      <c r="R10" s="85">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="43">
+        <v>1</v>
+      </c>
+      <c r="K11" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="P11" s="86" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q11" s="87">
+        <v>50</v>
+      </c>
+      <c r="R11" s="88">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="97"/>
+      <c r="C12" s="97"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="97"/>
+      <c r="F12" s="97"/>
+      <c r="G12" s="97"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="43">
+        <v>1</v>
+      </c>
+      <c r="K12" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+    </row>
+    <row r="13" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="60" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="59" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="35"/>
+      <c r="J13" s="43">
+        <v>1</v>
+      </c>
+      <c r="K13" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+    </row>
+    <row r="14" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="22"/>
+      <c r="B14" s="90"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="37"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="33"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+    </row>
+    <row r="15" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="56"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="43"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+    </row>
+    <row r="16" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="29"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+    </row>
+    <row r="17" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="29"/>
+      <c r="I17" s="35"/>
+      <c r="J17" s="43"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+    </row>
+    <row r="18" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="36"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="43"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+    </row>
+    <row r="19" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="32"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="I19" s="35"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+    </row>
+    <row r="20" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="32"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+    </row>
+    <row r="21" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="43"/>
+      <c r="K21" s="43"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+    </row>
+    <row r="22" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="32"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="43"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+    </row>
+    <row r="23" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="32"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="43"/>
+      <c r="K23" s="43"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
+    </row>
+    <row r="24" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="32"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="43"/>
+      <c r="K24" s="43"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+    </row>
+    <row r="25" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="32"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="43"/>
+      <c r="K25" s="43"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+    </row>
+    <row r="26" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="I26" s="35"/>
+      <c r="J26" s="43"/>
+      <c r="K26" s="43"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+    </row>
+    <row r="27" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="I27" s="35"/>
+      <c r="J27" s="43"/>
+      <c r="K27" s="43"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="22"/>
+    </row>
+    <row r="28" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="96" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="43"/>
+      <c r="K28" s="43"/>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+    </row>
+    <row r="29" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="54" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" s="35"/>
+      <c r="J29" s="43"/>
+      <c r="K29" s="43"/>
+      <c r="L29" s="22"/>
+      <c r="M29" s="22"/>
+    </row>
+    <row r="30" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="41">
+        <v>1</v>
+      </c>
+      <c r="B30" s="52"/>
+      <c r="C30" s="90">
+        <v>5</v>
+      </c>
+      <c r="D30" s="50">
+        <v>5</v>
+      </c>
+      <c r="E30" s="49" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30" s="47"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="43"/>
+      <c r="K30" s="43"/>
+      <c r="L30" s="22"/>
+      <c r="M30" s="22"/>
+    </row>
+    <row r="31" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="41"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="45"/>
+      <c r="G31" s="44"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="43"/>
+      <c r="K31" s="33"/>
+      <c r="L31" s="22"/>
+      <c r="M31" s="22"/>
+    </row>
+    <row r="32" spans="1:13" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="41"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="42"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="34"/>
+      <c r="K32" s="33"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+    </row>
+    <row r="33" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="41"/>
+      <c r="B33" s="40"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="29"/>
+      <c r="I33" s="35"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="38"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+    </row>
+    <row r="34" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="32"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="36"/>
+      <c r="I34" s="35"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="33"/>
+      <c r="L34" s="22"/>
+      <c r="M34" s="22"/>
+    </row>
+    <row r="35" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="32"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="34"/>
+      <c r="K35" s="33"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="22"/>
+    </row>
+    <row r="36" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="32"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="I36" s="35"/>
+      <c r="J36" s="34"/>
+      <c r="K36" s="33"/>
+      <c r="L36" s="22"/>
+      <c r="M36" s="22"/>
+    </row>
+    <row r="37" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="32"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="K37" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="L37" s="22">
+        <f>SUM(L2:L36)</f>
+        <v>23</v>
+      </c>
+      <c r="M37" s="22">
+        <f>SUM(M2:M36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="32"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+    </row>
+    <row r="39" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="32"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+    </row>
+    <row r="40" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="32"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+    </row>
+    <row r="41" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="21"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+    </row>
+    <row r="42" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="21"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="N42" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="O42" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="P42" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q42" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="R42" s="30" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="21"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="N43" s="98">
+        <v>1</v>
+      </c>
+      <c r="O43" s="25">
+        <f>VLOOKUP(P43,$I$2:$L$36,4,FALSE)</f>
+        <v>3</v>
+      </c>
+      <c r="P43" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q43" s="24" t="str">
+        <f>VLOOKUP(P43,$I$2:$L$36,3,FALSE)</f>
+        <v>nabil</v>
+      </c>
+      <c r="R43" s="101" t="e">
+        <f>SUM(O43:O47)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="21"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="N44" s="99"/>
+      <c r="O44" s="25" t="e">
+        <f t="shared" ref="O44:O68" si="0">VLOOKUP(P44,$I$3:$L$36,4,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P44" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q44" s="24" t="e">
+        <f t="shared" ref="Q44:Q68" si="1">VLOOKUP(P44,$I$3:$L$36,3,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R44" s="101"/>
+    </row>
+    <row r="45" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="21"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="N45" s="99"/>
+      <c r="O45" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P45" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q45" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R45" s="101"/>
+    </row>
+    <row r="46" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="N46" s="99"/>
+      <c r="O46" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P46" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q46" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R46" s="101"/>
+    </row>
+    <row r="47" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="21"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="N47" s="99"/>
+      <c r="O47" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P47" s="35" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q47" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R47" s="101"/>
+    </row>
+    <row r="48" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="21"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="21"/>
+      <c r="N48" s="98">
+        <v>2</v>
+      </c>
+      <c r="O48" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P48" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q48" s="28" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R48" s="103" t="e">
+        <f>SUM(O48:O49)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="21"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="21"/>
+      <c r="D49" s="21"/>
+      <c r="N49" s="99"/>
+      <c r="O49" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P49" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q49" s="28" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R49" s="103"/>
+    </row>
+    <row r="50" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="21"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="21"/>
+      <c r="D50" s="21"/>
+      <c r="N50" s="92">
+        <v>3</v>
+      </c>
+      <c r="O50" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P50" s="24"/>
+      <c r="Q50" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R50" s="89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="21"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="21"/>
+      <c r="D51" s="21"/>
+      <c r="N51" s="104">
+        <v>4</v>
+      </c>
+      <c r="O51" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P51" s="24"/>
+      <c r="Q51" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R51" s="106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="21"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="N52" s="105"/>
+      <c r="O52" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P52" s="24"/>
+      <c r="Q52" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R52" s="101"/>
+    </row>
+    <row r="53" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="21"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
+      <c r="N53" s="105"/>
+      <c r="O53" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P53" s="24"/>
+      <c r="Q53" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R53" s="101"/>
+    </row>
+    <row r="54" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="21"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="21"/>
+      <c r="D54" s="21"/>
+      <c r="N54" s="105"/>
+      <c r="O54" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P54" s="24"/>
+      <c r="Q54" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R54" s="101"/>
+    </row>
+    <row r="55" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="21"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="21"/>
+      <c r="N55" s="105"/>
+      <c r="O55" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P55" s="24"/>
+      <c r="Q55" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R55" s="101"/>
+    </row>
+    <row r="56" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="21"/>
+      <c r="B56" s="21"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="21"/>
+      <c r="N56" s="105"/>
+      <c r="O56" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P56" s="24"/>
+      <c r="Q56" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R56" s="101"/>
+    </row>
+    <row r="57" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="21"/>
+      <c r="B57" s="21"/>
+      <c r="C57" s="21"/>
+      <c r="D57" s="21"/>
+      <c r="N57" s="105"/>
+      <c r="O57" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P57" s="24"/>
+      <c r="Q57" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R57" s="101"/>
+    </row>
+    <row r="58" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="21"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="21"/>
+      <c r="D58" s="21"/>
+      <c r="N58" s="105"/>
+      <c r="O58" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P58" s="24"/>
+      <c r="Q58" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R58" s="107"/>
+    </row>
+    <row r="59" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="21"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="21"/>
+      <c r="D59" s="21"/>
+      <c r="N59" s="104">
+        <v>5</v>
+      </c>
+      <c r="O59" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P59" s="24"/>
+      <c r="Q59" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R59" s="106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="21"/>
+      <c r="B60" s="21"/>
+      <c r="C60" s="21"/>
+      <c r="D60" s="21"/>
+      <c r="N60" s="105"/>
+      <c r="O60" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P60" s="24"/>
+      <c r="Q60" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R60" s="105"/>
+    </row>
+    <row r="61" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="21"/>
+      <c r="B61" s="21"/>
+      <c r="C61" s="21"/>
+      <c r="D61" s="21"/>
+      <c r="N61" s="105"/>
+      <c r="O61" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P61" s="24"/>
+      <c r="Q61" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R61" s="105"/>
+    </row>
+    <row r="62" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="21"/>
+      <c r="B62" s="21"/>
+      <c r="C62" s="21"/>
+      <c r="D62" s="21"/>
+      <c r="N62" s="105"/>
+      <c r="O62" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P62" s="24"/>
+      <c r="Q62" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R62" s="105"/>
+    </row>
+    <row r="63" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="21"/>
+      <c r="B63" s="21"/>
+      <c r="C63" s="21"/>
+      <c r="D63" s="21"/>
+      <c r="N63" s="108"/>
+      <c r="O63" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P63" s="24"/>
+      <c r="Q63" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R63" s="108"/>
+    </row>
+    <row r="64" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="21"/>
+      <c r="B64" s="21"/>
+      <c r="C64" s="21"/>
+      <c r="D64" s="21"/>
+      <c r="N64" s="104">
+        <v>6</v>
+      </c>
+      <c r="O64" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P64" s="35" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q64" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R64" s="106" t="e">
+        <f>SUM(O64:O68)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="21"/>
+      <c r="B65" s="21"/>
+      <c r="C65" s="21"/>
+      <c r="D65" s="21"/>
+      <c r="N65" s="105"/>
+      <c r="O65" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P65" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q65" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R65" s="105"/>
+    </row>
+    <row r="66" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="21"/>
+      <c r="B66" s="21"/>
+      <c r="C66" s="21"/>
+      <c r="D66" s="21"/>
+      <c r="N66" s="105"/>
+      <c r="O66" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P66" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q66" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R66" s="105"/>
+    </row>
+    <row r="67" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="21"/>
+      <c r="B67" s="21"/>
+      <c r="C67" s="21"/>
+      <c r="D67" s="21"/>
+      <c r="N67" s="105"/>
+      <c r="O67" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P67" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q67" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R67" s="105"/>
+    </row>
+    <row r="68" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="21"/>
+      <c r="B68" s="21"/>
+      <c r="C68" s="21"/>
+      <c r="D68" s="21"/>
+      <c r="N68" s="108"/>
+      <c r="O68" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P68" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q68" s="24" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="R68" s="108"/>
+    </row>
+    <row r="69" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="21"/>
+      <c r="B69" s="21"/>
+      <c r="C69" s="21"/>
+      <c r="D69" s="21"/>
+      <c r="P69" s="24"/>
+      <c r="Q69" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="R69" s="22" t="e">
+        <f>SUM(R43:R68)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="21"/>
+      <c r="B70" s="21"/>
+      <c r="C70" s="21"/>
+      <c r="D70" s="21"/>
+    </row>
+    <row r="71" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="21"/>
+      <c r="B71" s="21"/>
+      <c r="C71" s="21"/>
+      <c r="D71" s="21"/>
+    </row>
+    <row r="72" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="21"/>
+      <c r="B72" s="21"/>
+      <c r="C72" s="21"/>
+      <c r="D72" s="21"/>
+    </row>
+    <row r="73" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="21"/>
+      <c r="B73" s="21"/>
+      <c r="C73" s="21"/>
+      <c r="D73" s="21"/>
+    </row>
+    <row r="74" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="21"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="21"/>
+    </row>
+    <row r="75" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="21"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="21"/>
+    </row>
+    <row r="76" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="21"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="21"/>
+    </row>
+    <row r="77" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="21"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+    </row>
+    <row r="78" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="21"/>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+    </row>
+    <row r="79" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="21"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="21"/>
+      <c r="D79" s="21"/>
+    </row>
+    <row r="80" spans="1:18" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="21"/>
+      <c r="B80" s="21"/>
+      <c r="C80" s="21"/>
+      <c r="D80" s="21"/>
+    </row>
+    <row r="81" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="21"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="21"/>
+      <c r="D81" s="21"/>
+    </row>
+    <row r="82" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="21"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="21"/>
+    </row>
+    <row r="83" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="21"/>
+      <c r="B83" s="21"/>
+      <c r="C83" s="21"/>
+      <c r="D83" s="21"/>
+    </row>
+    <row r="84" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="21"/>
+      <c r="B84" s="21"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="21"/>
+    </row>
+    <row r="85" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="21"/>
+      <c r="B85" s="21"/>
+      <c r="C85" s="21"/>
+      <c r="D85" s="21"/>
+    </row>
+    <row r="86" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="21"/>
+      <c r="B86" s="21"/>
+      <c r="C86" s="21"/>
+      <c r="D86" s="21"/>
+    </row>
+    <row r="87" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="21"/>
+      <c r="B87" s="21"/>
+      <c r="C87" s="21"/>
+      <c r="D87" s="21"/>
+    </row>
+    <row r="88" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="21"/>
+      <c r="B88" s="21"/>
+      <c r="C88" s="21"/>
+      <c r="D88" s="21"/>
+    </row>
+    <row r="89" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="21"/>
+      <c r="B89" s="21"/>
+      <c r="C89" s="21"/>
+      <c r="D89" s="21"/>
+    </row>
+    <row r="90" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="21"/>
+      <c r="B90" s="21"/>
+      <c r="C90" s="21"/>
+      <c r="D90" s="21"/>
+    </row>
+    <row r="91" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="21"/>
+      <c r="B91" s="21"/>
+      <c r="C91" s="21"/>
+      <c r="D91" s="21"/>
+    </row>
+    <row r="92" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="21"/>
+      <c r="B92" s="21"/>
+      <c r="C92" s="21"/>
+      <c r="D92" s="21"/>
+    </row>
+    <row r="93" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="21"/>
+      <c r="B93" s="21"/>
+      <c r="C93" s="21"/>
+      <c r="D93" s="21"/>
+    </row>
+    <row r="94" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="21"/>
+      <c r="B94" s="21"/>
+      <c r="C94" s="21"/>
+      <c r="D94" s="21"/>
+    </row>
+    <row r="95" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="21"/>
+      <c r="B95" s="21"/>
+      <c r="C95" s="21"/>
+      <c r="D95" s="21"/>
+    </row>
+    <row r="96" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="21"/>
+      <c r="B96" s="21"/>
+      <c r="C96" s="21"/>
+      <c r="D96" s="21"/>
+    </row>
+    <row r="97" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="21"/>
+      <c r="B97" s="21"/>
+      <c r="C97" s="21"/>
+      <c r="D97" s="21"/>
+    </row>
+    <row r="98" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="21"/>
+      <c r="B98" s="21"/>
+      <c r="C98" s="21"/>
+      <c r="D98" s="21"/>
+    </row>
+    <row r="99" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="21"/>
+      <c r="B99" s="21"/>
+      <c r="C99" s="21"/>
+      <c r="D99" s="21"/>
+    </row>
+    <row r="100" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="21"/>
+      <c r="B100" s="21"/>
+      <c r="C100" s="21"/>
+      <c r="D100" s="21"/>
+    </row>
+    <row r="101" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="21"/>
+      <c r="B101" s="21"/>
+      <c r="C101" s="21"/>
+      <c r="D101" s="21"/>
+    </row>
+    <row r="102" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="21"/>
+      <c r="B102" s="21"/>
+      <c r="C102" s="21"/>
+      <c r="D102" s="21"/>
+    </row>
+    <row r="103" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="21"/>
+      <c r="B103" s="21"/>
+      <c r="C103" s="21"/>
+      <c r="D103" s="21"/>
+    </row>
+    <row r="104" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="21"/>
+      <c r="B104" s="21"/>
+      <c r="C104" s="21"/>
+      <c r="D104" s="21"/>
+    </row>
+    <row r="105" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="21"/>
+      <c r="B105" s="21"/>
+      <c r="C105" s="21"/>
+      <c r="D105" s="21"/>
+    </row>
+    <row r="106" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="21"/>
+      <c r="B106" s="21"/>
+      <c r="C106" s="21"/>
+      <c r="D106" s="21"/>
+    </row>
+    <row r="107" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="21"/>
+      <c r="B107" s="21"/>
+      <c r="C107" s="21"/>
+      <c r="D107" s="21"/>
+    </row>
+    <row r="108" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="21"/>
+      <c r="B108" s="21"/>
+      <c r="C108" s="21"/>
+      <c r="D108" s="21"/>
+    </row>
+    <row r="109" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="21"/>
+      <c r="B109" s="21"/>
+      <c r="C109" s="21"/>
+      <c r="D109" s="21"/>
+    </row>
+    <row r="110" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="21"/>
+      <c r="B110" s="21"/>
+      <c r="C110" s="21"/>
+      <c r="D110" s="21"/>
+    </row>
+    <row r="111" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="21"/>
+      <c r="B111" s="21"/>
+      <c r="C111" s="21"/>
+      <c r="D111" s="21"/>
+    </row>
+    <row r="112" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="21"/>
+      <c r="B112" s="21"/>
+      <c r="C112" s="21"/>
+      <c r="D112" s="21"/>
+    </row>
+    <row r="113" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="21"/>
+      <c r="B113" s="21"/>
+      <c r="C113" s="21"/>
+      <c r="D113" s="21"/>
+    </row>
+    <row r="114" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="21"/>
+      <c r="B114" s="21"/>
+      <c r="C114" s="21"/>
+      <c r="D114" s="21"/>
+    </row>
+    <row r="115" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="21"/>
+      <c r="B115" s="21"/>
+      <c r="C115" s="21"/>
+      <c r="D115" s="21"/>
+    </row>
+    <row r="116" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="21"/>
+      <c r="B116" s="21"/>
+      <c r="C116" s="21"/>
+      <c r="D116" s="21"/>
+    </row>
+    <row r="117" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="21"/>
+      <c r="B117" s="21"/>
+      <c r="C117" s="21"/>
+      <c r="D117" s="21"/>
+    </row>
+    <row r="118" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="21"/>
+      <c r="B118" s="21"/>
+      <c r="C118" s="21"/>
+      <c r="D118" s="21"/>
+    </row>
+    <row r="119" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="21"/>
+      <c r="B119" s="21"/>
+      <c r="C119" s="21"/>
+      <c r="D119" s="21"/>
+    </row>
+    <row r="120" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="21"/>
+      <c r="B120" s="21"/>
+      <c r="C120" s="21"/>
+      <c r="D120" s="21"/>
+    </row>
+    <row r="121" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="21"/>
+      <c r="B121" s="21"/>
+      <c r="C121" s="21"/>
+      <c r="D121" s="21"/>
+    </row>
+    <row r="122" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="21"/>
+      <c r="B122" s="21"/>
+      <c r="C122" s="21"/>
+      <c r="D122" s="21"/>
+    </row>
+    <row r="123" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="21"/>
+      <c r="B123" s="21"/>
+      <c r="C123" s="21"/>
+      <c r="D123" s="21"/>
+    </row>
+    <row r="124" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="21"/>
+      <c r="B124" s="21"/>
+      <c r="C124" s="21"/>
+      <c r="D124" s="21"/>
+    </row>
+    <row r="125" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="21"/>
+      <c r="B125" s="21"/>
+      <c r="C125" s="21"/>
+      <c r="D125" s="21"/>
+    </row>
+    <row r="126" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="21"/>
+      <c r="B126" s="21"/>
+      <c r="C126" s="21"/>
+      <c r="D126" s="21"/>
+    </row>
+    <row r="127" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="21"/>
+      <c r="B127" s="21"/>
+      <c r="C127" s="21"/>
+      <c r="D127" s="21"/>
+    </row>
+    <row r="128" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="21"/>
+      <c r="B128" s="21"/>
+      <c r="C128" s="21"/>
+      <c r="D128" s="21"/>
+    </row>
+    <row r="129" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="21"/>
+      <c r="B129" s="21"/>
+      <c r="C129" s="21"/>
+      <c r="D129" s="21"/>
+    </row>
+    <row r="130" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="21"/>
+      <c r="B130" s="21"/>
+      <c r="C130" s="21"/>
+      <c r="D130" s="21"/>
+    </row>
+    <row r="131" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="21"/>
+      <c r="B131" s="21"/>
+      <c r="C131" s="21"/>
+      <c r="D131" s="21"/>
+    </row>
+    <row r="132" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="21"/>
+      <c r="B132" s="21"/>
+      <c r="C132" s="21"/>
+      <c r="D132" s="21"/>
+    </row>
+    <row r="133" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="21"/>
+      <c r="B133" s="21"/>
+      <c r="C133" s="21"/>
+      <c r="D133" s="21"/>
+    </row>
+    <row r="134" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="21"/>
+      <c r="B134" s="21"/>
+      <c r="C134" s="21"/>
+      <c r="D134" s="21"/>
+    </row>
+    <row r="135" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="21"/>
+      <c r="B135" s="21"/>
+      <c r="C135" s="21"/>
+      <c r="D135" s="21"/>
+    </row>
+    <row r="136" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="21"/>
+      <c r="B136" s="21"/>
+      <c r="C136" s="21"/>
+      <c r="D136" s="21"/>
+    </row>
+    <row r="137" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="21"/>
+      <c r="B137" s="21"/>
+      <c r="C137" s="21"/>
+      <c r="D137" s="21"/>
+    </row>
+    <row r="138" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="21"/>
+      <c r="B138" s="21"/>
+      <c r="C138" s="21"/>
+      <c r="D138" s="21"/>
+    </row>
+    <row r="139" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="21"/>
+      <c r="B139" s="21"/>
+      <c r="C139" s="21"/>
+      <c r="D139" s="21"/>
+    </row>
+    <row r="140" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="21"/>
+      <c r="B140" s="21"/>
+      <c r="C140" s="21"/>
+      <c r="D140" s="21"/>
+    </row>
+    <row r="141" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="21"/>
+      <c r="B141" s="21"/>
+      <c r="C141" s="21"/>
+      <c r="D141" s="21"/>
+    </row>
+    <row r="142" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="21"/>
+      <c r="B142" s="21"/>
+      <c r="C142" s="21"/>
+      <c r="D142" s="21"/>
+    </row>
+    <row r="143" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="21"/>
+      <c r="B143" s="21"/>
+      <c r="C143" s="21"/>
+      <c r="D143" s="21"/>
+    </row>
+    <row r="144" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="21"/>
+      <c r="B144" s="21"/>
+      <c r="C144" s="21"/>
+      <c r="D144" s="21"/>
+    </row>
+    <row r="145" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="21"/>
+      <c r="B145" s="21"/>
+      <c r="C145" s="21"/>
+      <c r="D145" s="21"/>
+    </row>
+    <row r="146" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="21"/>
+      <c r="B146" s="21"/>
+      <c r="C146" s="21"/>
+      <c r="D146" s="21"/>
+    </row>
+    <row r="147" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="21"/>
+      <c r="B147" s="21"/>
+      <c r="C147" s="21"/>
+      <c r="D147" s="21"/>
+    </row>
+    <row r="148" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="21"/>
+      <c r="B148" s="21"/>
+      <c r="C148" s="21"/>
+      <c r="D148" s="21"/>
+    </row>
+    <row r="149" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="21"/>
+      <c r="B149" s="21"/>
+      <c r="C149" s="21"/>
+      <c r="D149" s="21"/>
+    </row>
+    <row r="150" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="21"/>
+      <c r="B150" s="21"/>
+      <c r="C150" s="21"/>
+      <c r="D150" s="21"/>
+    </row>
+    <row r="151" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="21"/>
+      <c r="B151" s="21"/>
+      <c r="C151" s="21"/>
+      <c r="D151" s="21"/>
+    </row>
+    <row r="152" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="21"/>
+      <c r="B152" s="21"/>
+      <c r="C152" s="21"/>
+      <c r="D152" s="21"/>
+    </row>
+    <row r="153" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="21"/>
+      <c r="B153" s="21"/>
+      <c r="C153" s="21"/>
+      <c r="D153" s="21"/>
+    </row>
+    <row r="154" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="21"/>
+      <c r="B154" s="21"/>
+      <c r="C154" s="21"/>
+      <c r="D154" s="21"/>
+    </row>
+    <row r="155" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="21"/>
+      <c r="B155" s="21"/>
+      <c r="C155" s="21"/>
+      <c r="D155" s="21"/>
+    </row>
+    <row r="156" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="21"/>
+      <c r="B156" s="21"/>
+      <c r="C156" s="21"/>
+      <c r="D156" s="21"/>
+    </row>
+    <row r="157" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="21"/>
+      <c r="B157" s="21"/>
+      <c r="C157" s="21"/>
+      <c r="D157" s="21"/>
+    </row>
+    <row r="158" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="21"/>
+      <c r="B158" s="21"/>
+      <c r="C158" s="21"/>
+      <c r="D158" s="21"/>
+    </row>
+    <row r="159" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="21"/>
+      <c r="B159" s="21"/>
+      <c r="C159" s="21"/>
+      <c r="D159" s="21"/>
+    </row>
+    <row r="160" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="21"/>
+      <c r="B160" s="21"/>
+      <c r="C160" s="21"/>
+      <c r="D160" s="21"/>
+    </row>
+    <row r="161" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="21"/>
+      <c r="B161" s="21"/>
+      <c r="C161" s="21"/>
+      <c r="D161" s="21"/>
+    </row>
+    <row r="162" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="21"/>
+      <c r="B162" s="21"/>
+      <c r="C162" s="21"/>
+      <c r="D162" s="21"/>
+    </row>
+    <row r="163" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="21"/>
+      <c r="B163" s="21"/>
+      <c r="C163" s="21"/>
+      <c r="D163" s="21"/>
+    </row>
+    <row r="164" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="21"/>
+      <c r="B164" s="21"/>
+      <c r="C164" s="21"/>
+      <c r="D164" s="21"/>
+    </row>
+    <row r="165" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="21"/>
+      <c r="B165" s="21"/>
+      <c r="C165" s="21"/>
+      <c r="D165" s="21"/>
+    </row>
+    <row r="166" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="21"/>
+      <c r="B166" s="21"/>
+      <c r="C166" s="21"/>
+      <c r="D166" s="21"/>
+    </row>
+    <row r="167" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="21"/>
+      <c r="B167" s="21"/>
+      <c r="C167" s="21"/>
+      <c r="D167" s="21"/>
+    </row>
+    <row r="168" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="21"/>
+      <c r="B168" s="21"/>
+      <c r="C168" s="21"/>
+      <c r="D168" s="21"/>
+    </row>
+    <row r="169" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="21"/>
+      <c r="B169" s="21"/>
+      <c r="C169" s="21"/>
+      <c r="D169" s="21"/>
+    </row>
+    <row r="170" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="21"/>
+      <c r="B170" s="21"/>
+      <c r="C170" s="21"/>
+      <c r="D170" s="21"/>
+    </row>
+    <row r="171" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="21"/>
+      <c r="B171" s="21"/>
+      <c r="C171" s="21"/>
+      <c r="D171" s="21"/>
+    </row>
+    <row r="172" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="21"/>
+      <c r="B172" s="21"/>
+      <c r="C172" s="21"/>
+      <c r="D172" s="21"/>
+    </row>
+    <row r="173" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="21"/>
+      <c r="B173" s="21"/>
+      <c r="C173" s="21"/>
+      <c r="D173" s="21"/>
+    </row>
+    <row r="174" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="21"/>
+      <c r="B174" s="21"/>
+      <c r="C174" s="21"/>
+      <c r="D174" s="21"/>
+    </row>
+    <row r="175" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="21"/>
+      <c r="B175" s="21"/>
+      <c r="C175" s="21"/>
+      <c r="D175" s="21"/>
+    </row>
+    <row r="176" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="21"/>
+      <c r="B176" s="21"/>
+      <c r="C176" s="21"/>
+      <c r="D176" s="21"/>
+    </row>
+    <row r="177" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="21"/>
+      <c r="B177" s="21"/>
+      <c r="C177" s="21"/>
+      <c r="D177" s="21"/>
+    </row>
+    <row r="178" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="21"/>
+      <c r="B178" s="21"/>
+      <c r="C178" s="21"/>
+      <c r="D178" s="21"/>
+    </row>
+    <row r="179" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="21"/>
+      <c r="B179" s="21"/>
+      <c r="C179" s="21"/>
+      <c r="D179" s="21"/>
+    </row>
+    <row r="180" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="21"/>
+      <c r="B180" s="21"/>
+      <c r="C180" s="21"/>
+      <c r="D180" s="21"/>
+    </row>
+    <row r="181" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="21"/>
+      <c r="B181" s="21"/>
+      <c r="C181" s="21"/>
+      <c r="D181" s="21"/>
+    </row>
+    <row r="182" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="21"/>
+      <c r="B182" s="21"/>
+      <c r="C182" s="21"/>
+      <c r="D182" s="21"/>
+    </row>
+    <row r="183" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="21"/>
+      <c r="B183" s="21"/>
+      <c r="C183" s="21"/>
+      <c r="D183" s="21"/>
+    </row>
+    <row r="184" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="21"/>
+      <c r="B184" s="21"/>
+      <c r="C184" s="21"/>
+      <c r="D184" s="21"/>
+    </row>
+    <row r="185" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="21"/>
+      <c r="B185" s="21"/>
+      <c r="C185" s="21"/>
+      <c r="D185" s="21"/>
+    </row>
+    <row r="186" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="21"/>
+      <c r="B186" s="21"/>
+      <c r="C186" s="21"/>
+      <c r="D186" s="21"/>
+    </row>
+    <row r="187" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="21"/>
+      <c r="B187" s="21"/>
+      <c r="C187" s="21"/>
+      <c r="D187" s="21"/>
+    </row>
+    <row r="188" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="21"/>
+      <c r="B188" s="21"/>
+      <c r="C188" s="21"/>
+      <c r="D188" s="21"/>
+    </row>
+    <row r="189" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="21"/>
+      <c r="B189" s="21"/>
+      <c r="C189" s="21"/>
+      <c r="D189" s="21"/>
+    </row>
+    <row r="190" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="21"/>
+      <c r="B190" s="21"/>
+      <c r="C190" s="21"/>
+      <c r="D190" s="21"/>
+    </row>
+    <row r="191" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="21"/>
+      <c r="B191" s="21"/>
+      <c r="C191" s="21"/>
+      <c r="D191" s="21"/>
+    </row>
+    <row r="192" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="21"/>
+      <c r="B192" s="21"/>
+      <c r="C192" s="21"/>
+      <c r="D192" s="21"/>
+    </row>
+    <row r="193" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="21"/>
+      <c r="B193" s="21"/>
+      <c r="C193" s="21"/>
+      <c r="D193" s="21"/>
+    </row>
+    <row r="194" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="21"/>
+      <c r="B194" s="21"/>
+      <c r="C194" s="21"/>
+      <c r="D194" s="21"/>
+    </row>
+    <row r="195" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="21"/>
+      <c r="B195" s="21"/>
+      <c r="C195" s="21"/>
+      <c r="D195" s="21"/>
+    </row>
+    <row r="196" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="21"/>
+      <c r="B196" s="21"/>
+      <c r="C196" s="21"/>
+      <c r="D196" s="21"/>
+    </row>
+    <row r="197" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="21"/>
+      <c r="B197" s="21"/>
+      <c r="C197" s="21"/>
+      <c r="D197" s="21"/>
+    </row>
+    <row r="198" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="21"/>
+      <c r="B198" s="21"/>
+      <c r="C198" s="21"/>
+      <c r="D198" s="21"/>
+    </row>
+    <row r="199" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="21"/>
+      <c r="B199" s="21"/>
+      <c r="C199" s="21"/>
+      <c r="D199" s="21"/>
+    </row>
+    <row r="200" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="21"/>
+      <c r="B200" s="21"/>
+      <c r="C200" s="21"/>
+      <c r="D200" s="21"/>
+    </row>
+    <row r="201" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="21"/>
+      <c r="B201" s="21"/>
+      <c r="C201" s="21"/>
+      <c r="D201" s="21"/>
+    </row>
+    <row r="202" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="21"/>
+      <c r="B202" s="21"/>
+      <c r="C202" s="21"/>
+      <c r="D202" s="21"/>
+    </row>
+    <row r="203" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="21"/>
+      <c r="B203" s="21"/>
+      <c r="C203" s="21"/>
+      <c r="D203" s="21"/>
+    </row>
+    <row r="204" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="21"/>
+      <c r="B204" s="21"/>
+      <c r="C204" s="21"/>
+      <c r="D204" s="21"/>
+    </row>
+    <row r="205" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="21"/>
+      <c r="B205" s="21"/>
+      <c r="C205" s="21"/>
+      <c r="D205" s="21"/>
+    </row>
+    <row r="206" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="21"/>
+      <c r="B206" s="21"/>
+      <c r="C206" s="21"/>
+      <c r="D206" s="21"/>
+    </row>
+    <row r="207" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="21"/>
+      <c r="B207" s="21"/>
+      <c r="C207" s="21"/>
+      <c r="D207" s="21"/>
+    </row>
+    <row r="208" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="21"/>
+      <c r="B208" s="21"/>
+      <c r="C208" s="21"/>
+      <c r="D208" s="21"/>
+    </row>
+    <row r="209" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="21"/>
+      <c r="B209" s="21"/>
+      <c r="C209" s="21"/>
+      <c r="D209" s="21"/>
+    </row>
+    <row r="210" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="21"/>
+      <c r="B210" s="21"/>
+      <c r="C210" s="21"/>
+      <c r="D210" s="21"/>
+    </row>
+    <row r="211" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="21"/>
+      <c r="B211" s="21"/>
+      <c r="C211" s="21"/>
+      <c r="D211" s="21"/>
+    </row>
+    <row r="212" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="21"/>
+      <c r="B212" s="21"/>
+      <c r="C212" s="21"/>
+      <c r="D212" s="21"/>
+    </row>
+    <row r="213" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A213" s="21"/>
+      <c r="B213" s="21"/>
+      <c r="C213" s="21"/>
+      <c r="D213" s="21"/>
+    </row>
+    <row r="214" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A214" s="21"/>
+      <c r="B214" s="21"/>
+      <c r="C214" s="21"/>
+      <c r="D214" s="21"/>
+    </row>
+    <row r="215" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="21"/>
+      <c r="B215" s="21"/>
+      <c r="C215" s="21"/>
+      <c r="D215" s="21"/>
+    </row>
+    <row r="216" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="21"/>
+      <c r="B216" s="21"/>
+      <c r="C216" s="21"/>
+      <c r="D216" s="21"/>
+    </row>
+    <row r="217" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="21"/>
+      <c r="B217" s="21"/>
+      <c r="C217" s="21"/>
+      <c r="D217" s="21"/>
+    </row>
+    <row r="218" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="21"/>
+      <c r="B218" s="21"/>
+      <c r="C218" s="21"/>
+      <c r="D218" s="21"/>
+    </row>
+    <row r="219" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="21"/>
+      <c r="B219" s="21"/>
+      <c r="C219" s="21"/>
+      <c r="D219" s="21"/>
+    </row>
+    <row r="220" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="21"/>
+      <c r="B220" s="21"/>
+      <c r="C220" s="21"/>
+      <c r="D220" s="21"/>
+    </row>
+    <row r="221" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="21"/>
+      <c r="B221" s="21"/>
+      <c r="C221" s="21"/>
+      <c r="D221" s="21"/>
+    </row>
+    <row r="222" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="21"/>
+      <c r="B222" s="21"/>
+      <c r="C222" s="21"/>
+      <c r="D222" s="21"/>
+    </row>
+    <row r="223" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="21"/>
+      <c r="B223" s="21"/>
+      <c r="C223" s="21"/>
+      <c r="D223" s="21"/>
+    </row>
+    <row r="224" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A224" s="21"/>
+      <c r="B224" s="21"/>
+      <c r="C224" s="21"/>
+      <c r="D224" s="21"/>
+    </row>
+    <row r="225" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="21"/>
+      <c r="B225" s="21"/>
+      <c r="C225" s="21"/>
+      <c r="D225" s="21"/>
+    </row>
+    <row r="226" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="21"/>
+      <c r="B226" s="21"/>
+      <c r="C226" s="21"/>
+      <c r="D226" s="21"/>
+    </row>
+    <row r="227" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="21"/>
+      <c r="B227" s="21"/>
+      <c r="C227" s="21"/>
+      <c r="D227" s="21"/>
+    </row>
+    <row r="228" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A228" s="21"/>
+      <c r="B228" s="21"/>
+      <c r="C228" s="21"/>
+      <c r="D228" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="N51:N58"/>
+    <mergeCell ref="R51:R58"/>
+    <mergeCell ref="N59:N63"/>
+    <mergeCell ref="R59:R63"/>
+    <mergeCell ref="N64:N68"/>
+    <mergeCell ref="R64:R68"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="N43:N47"/>
+    <mergeCell ref="R43:R47"/>
+    <mergeCell ref="N48:N49"/>
+    <mergeCell ref="R48:R49"/>
+  </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F14:F25 F30:F40" xr:uid="{67546FD1-F383-41E0-BB8B-2F4BEECE4BCF}">
+      <formula1>"Avoid,Mitigate,Accept"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="portrait"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>